<commit_message>
Carry the Pi's supply and the reader's cable in kind
Both are already on hand, so the power supply row moves to "Already have"
and leaves the subtotal, and the USB-C to USB-A cable - which the table never
listed although it is the reader's only link to the Pi - joins as an in-kind
row. Subtotal $477.38, leaving $22.62 under the shipping plug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Materials-and-Cost-Table.xlsx
+++ b/docs/Materials-and-Cost-Table.xlsx
@@ -1544,19 +1544,23 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.1 V · 3 A · US plug · official</t>
+          <t xml:space="preserve">5.1 V · 3 A · USB-C · official</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.pishop.us/product/raspberry-pi-15w-power-supply-us-black/</t>
-        </is>
-      </c>
-      <c r="F13" s="2">
-        <v>8.8</v>
-      </c>
-      <c r="G13" s="2">
-        <v>8.8</v>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
@@ -1630,14 +1634,40 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="20"/>
+    <row r="16" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USB-C to USB-A cable</t>
+        </is>
+      </c>
+      <c r="C16" s="19">
+        <v>1</v>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≤ 1 ft · data-capable, not charge-only</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joins the reader's USB-C port to the Pi. It is the reader's only data and power link.</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B17" s="21"/>
@@ -1653,8 +1683,8 @@
         <v>12</v>
       </c>
       <c r="G18" s="34">
-        <f>SUM(G6,G7,G8,G10,G11,G12,G13,G15)</f>
-        <v>486.18</v>
+        <f>SUM(G6,G7,G8,G10,G11,G12,G15)</f>
+        <v>477.38</v>
       </c>
       <c r="H18" s="35"/>
     </row>
@@ -1673,7 +1703,7 @@
       </c>
       <c r="G20" s="27">
         <f>500-G18</f>
-        <v>13.82</v>
+        <v>22.62</v>
       </c>
       <c r="H20" s="28"/>
     </row>

</xml_diff>

<commit_message>
Carry the RTC's jumper wires in kind
The DS3231 breakout has no plug-in connector, so four female-to-female wires
are what join it to the Pi's header. They are already on hand, and so is the
microSD, which the table already carried in kind. The subtotal is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Materials-and-Cost-Table.xlsx
+++ b/docs/Materials-and-Cost-Table.xlsx
@@ -1669,14 +1669,40 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B17" s="21"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="26"/>
+    <row r="17" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Female-to-female jumper wires</t>
+        </is>
+      </c>
+      <c r="C17" s="22">
+        <v>4</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.54 mm Dupont · 20 cm</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wire the DS3231's VIN, GND, SDA and SCL to the Pi's GPIO header; the breakout has no plug-in connector.</t>
+        </is>
+      </c>
     </row>
     <row r="18" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="F18" s="6" t="s">

</xml_diff>

<commit_message>
Carry the boards' M2.5 mounting hardware in kind
Eight screws, nuts and standoffs - four for the Pi 4, four for the Hecto,
whose 4-40 holes M2.5 fits - are already on hand. The table had no empty
line left, so one is inserted above the last item and the totals block moves
down a row: its formulas, merged cells and calc chain move with it, and the
subtotal is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Materials-and-Cost-Table.xlsx
+++ b/docs/Materials-and-Cost-Table.xlsx
@@ -1253,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:H22"/>
+  <dimension ref="B2:H23"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1670,97 +1670,132 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2.5 screws, nuts and standoffs</t>
+        </is>
+      </c>
+      <c r="C17" s="19">
+        <v>8</v>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2.5 · nylon or brass · 4 for the Pi, 4 for the reader</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mount the Pi 4 (58 × 49 mm hole pattern) and the Hecto (4-40 holes, which M2.5 fits) to the base plate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Female-to-female jumper wires</t>
         </is>
       </c>
-      <c r="C17" s="22">
+      <c r="C18" s="22">
         <v>4</v>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2.54 mm Dupont · 20 cm</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
+      <c r="F18" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="G17" s="25" t="inlineStr">
+      <c r="G18" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="H17" s="26" t="inlineStr">
+      <c r="H18" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Wire the DS3231's VIN, GND, SDA and SCL to the Pi's GPIO header; the breakout has no plug-in connector.</t>
         </is>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F18" s="6" t="s">
+    <row r="19" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G18" s="34">
+      <c r="G19" s="34">
         <f>SUM(G6,G7,G8,G10,G11,G12,G15)</f>
         <v>477.38</v>
       </c>
-      <c r="H18" s="35"/>
-    </row>
-    <row r="19" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F19" s="7" t="s">
+      <c r="H19" s="35"/>
+    </row>
+    <row r="20" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F20" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G20" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="28"/>
-    </row>
-    <row r="20" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F20" s="8" t="s">
+      <c r="H20" s="28"/>
+    </row>
+    <row r="21" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F21" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G20" s="27">
-        <f>500-G18</f>
+      <c r="G21" s="27">
+        <f>500-G19</f>
         <v>22.62</v>
       </c>
-      <c r="H20" s="28"/>
-    </row>
-    <row r="21" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F21" s="9" t="s">
+      <c r="H21" s="28"/>
+    </row>
+    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F22" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="G22" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="H21" s="28"/>
-    </row>
-    <row r="22" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F22" s="10" t="s">
+      <c r="H22" s="28"/>
+    </row>
+    <row r="23" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F23" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="29">
-        <f>G18+G20</f>
+      <c r="G23" s="29">
+        <f>G19+G21</f>
         <v>500</v>
       </c>
-      <c r="H22" s="30"/>
+      <c r="H23" s="30"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="G18:H18"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="G4:H4"/>

</xml_diff>

<commit_message>
Add the enclosure and its cooling to the table
The enclosure is already printed and a 5 V fan run from the Pi's header is
already on hand, so both are carried in kind. The Pi 4 heatsink set is the
one thing bought, $2.95 at PiShop: the box is closed but for its rear vents,
and the fan only helps once the heat can leave the chips. Three rows are
inserted above the last item and the totals block moves to rows 22-26.
Subtotal $480.33, leaving $19.67 under the shipping plug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Materials-and-Cost-Table.xlsx
+++ b/docs/Materials-and-Cost-Table.xlsx
@@ -1253,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:H23"/>
+  <dimension ref="B2:H26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1705,97 +1705,198 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3D-printed enclosure</t>
+        </is>
+      </c>
+      <c r="C18" s="19">
+        <v>1</v>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printed body, panels and base plate</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Houses the Pi, reader, clock and antenna. Keep metal and cables out of the antenna's path through the front face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cooling fan</t>
+        </is>
+      </c>
+      <c r="C19" s="19">
+        <v>1</v>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 V, powered from the Pi's GPIO header</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already have</t>
+        </is>
+      </c>
+      <c r="H19" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moves the Pi's and the reader's heat out through the rear vents; the box is otherwise closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Raspberry Pi 4 heatsink set</t>
+        </is>
+      </c>
+      <c r="C20" s="19">
+        <v>1</v>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aluminium · 3 pieces (CPU, RAM, USB controller) · 3M 8810 thermal tape</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.pishop.us/product/aluminum-heatsink-for-raspberry-pi-4b-3-pack/</t>
+        </is>
+      </c>
+      <c r="F20" s="2">
+        <v>2.95</v>
+      </c>
+      <c r="G20" s="2">
+        <v>2.95</v>
+      </c>
+      <c r="H20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Pi 4 throttles when hot. The fan only helps if the heat can leave the chips first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Female-to-female jumper wires</t>
         </is>
       </c>
-      <c r="C18" s="22">
+      <c r="C21" s="22">
         <v>4</v>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2.54 mm Dupont · 20 cm</t>
         </is>
       </c>
-      <c r="E18" s="23" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="F18" s="24" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="G18" s="25" t="inlineStr">
+      <c r="G21" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Already have</t>
         </is>
       </c>
-      <c r="H18" s="26" t="inlineStr">
+      <c r="H21" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Wire the DS3231's VIN, GND, SDA and SCL to the Pi's GPIO header; the breakout has no plug-in connector.</t>
         </is>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F19" s="6" t="s">
+    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F22" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="34">
-        <f>SUM(G6,G7,G8,G10,G11,G12,G15)</f>
-        <v>477.38</v>
-      </c>
-      <c r="H19" s="35"/>
-    </row>
-    <row r="20" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F20" s="7" t="s">
+      <c r="G22" s="34">
+        <f>SUM(G6,G7,G8,G10,G11,G12,G15,G20)</f>
+        <v>480.33</v>
+      </c>
+      <c r="H22" s="35"/>
+    </row>
+    <row r="23" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F23" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="G23" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="28"/>
-    </row>
-    <row r="21" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F21" s="8" t="s">
+      <c r="H23" s="28"/>
+    </row>
+    <row r="24" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F24" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G21" s="27">
-        <f>500-G19</f>
-        <v>22.62</v>
-      </c>
-      <c r="H21" s="28"/>
-    </row>
-    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F22" s="9" t="s">
+      <c r="G24" s="27">
+        <f>500-G22</f>
+        <v>19.67</v>
+      </c>
+      <c r="H24" s="28"/>
+    </row>
+    <row r="25" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F25" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="27" t="s">
+      <c r="G25" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="H22" s="28"/>
-    </row>
-    <row r="23" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F23" s="10" t="s">
+      <c r="H25" s="28"/>
+    </row>
+    <row r="26" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="F26" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G23" s="29">
-        <f>G19+G21</f>
+      <c r="G26" s="29">
+        <f>G22+G24</f>
         <v>500</v>
       </c>
-      <c r="H23" s="30"/>
+      <c r="H26" s="30"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="G19:H19"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="G4:H4"/>

</xml_diff>